<commit_message>
Version 1.2 - Updated QA checklist
</commit_message>
<xml_diff>
--- a/QA-Checklist.xlsx
+++ b/QA-Checklist.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Studio-65_Share\Version-Control-Task\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5EC528E-6BFB-4CF0-9AE9-3F6E5961D034}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF938CB9-9342-408E-AF7E-51C68B0EEDC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="3975" windowWidth="10200" windowHeight="11625" xr2:uid="{1C972986-9CE9-4C10-A93D-84465225EB9F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{1C972986-9CE9-4C10-A93D-84465225EB9F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="21">
   <si>
     <t>Check ID</t>
   </si>
@@ -73,13 +73,28 @@
   </si>
   <si>
     <t>Login works with valid credentials</t>
+  </si>
+  <si>
+    <t>QA Checklist</t>
+  </si>
+  <si>
+    <t>Version: 1.2</t>
+  </si>
+  <si>
+    <t>CHK005</t>
+  </si>
+  <si>
+    <t>Forgot Password works</t>
+  </si>
+  <si>
+    <t>Password reset works</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -94,6 +109,17 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
     </font>
   </fonts>
   <fills count="2">
@@ -116,12 +142,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -438,82 +472,108 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D87CEDD4-D9A1-44A0-968B-EC502D218E10}">
-  <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="15.28515625" customWidth="1"/>
-    <col min="3" max="3" width="10.42578125" customWidth="1"/>
+    <col min="1" max="1" width="14.5703125" customWidth="1"/>
+    <col min="2" max="2" width="14.42578125" customWidth="1"/>
+    <col min="3" max="3" width="21" customWidth="1"/>
+    <col min="4" max="4" width="10.42578125" customWidth="1"/>
+    <col min="5" max="5" width="23.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:5">
+      <c r="A1" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:5" ht="30">
+      <c r="A2" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
+    <row r="3" spans="1:5" ht="30">
+      <c r="B3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="C3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
+    <row r="4" spans="1:5">
+      <c r="B4" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="C4" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="D4" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="E4" s="2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="90" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
+    <row r="5" spans="1:5" ht="30">
+      <c r="B5" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="C5" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="D5" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="E5" s="2" t="s">
         <v>15</v>
       </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="B6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="E7" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>